<commit_message>
I think it's final
</commit_message>
<xml_diff>
--- a/Список проверенных переводов.xlsx
+++ b/Список проверенных переводов.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Disposable\Desktop\СЦЕНАРИИ\В процессе\DanilChem\DBD_Localization\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4A6FD795-5EC2-446F-A589-B3B4B46B9123}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DB136566-3F14-46A5-897C-CD7E15AEECE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14016" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2139,7 +2139,7 @@
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="4" t="s">
+      <c r="A25" s="13" t="s">
         <v>68</v>
       </c>
       <c r="B25" s="2" t="s">
@@ -2159,7 +2159,7 @@
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
+      <c r="A26" s="13" t="s">
         <v>69</v>
       </c>
       <c r="B26" s="2" t="s">
@@ -2179,7 +2179,7 @@
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
+      <c r="A27" s="13" t="s">
         <v>70</v>
       </c>
       <c r="B27" s="2" t="s">
@@ -2199,7 +2199,7 @@
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
+      <c r="A28" s="13" t="s">
         <v>71</v>
       </c>
       <c r="B28" s="2" t="s">
@@ -2299,7 +2299,7 @@
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A33" s="4" t="s">
+      <c r="A33" s="13" t="s">
         <v>75</v>
       </c>
       <c r="B33" s="2" t="s">
@@ -2319,7 +2319,7 @@
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A34" s="4" t="s">
+      <c r="A34" s="13" t="s">
         <v>76</v>
       </c>
       <c r="B34" s="2" t="s">

</xml_diff>